<commit_message>
Example workbooks: restore Crop Planning Guide to original formatting; apply minimum row height to MB elevator without altering its fonts
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mb_primary_elevator_capacity_2025.xlsx
+++ b/textbook_examples/mb_primary_elevator_capacity_2025.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -143,44 +143,6 @@
       <sz val="8"/>
       <u val="single"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color indexed="8"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="10"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <sz val="10"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -701,7 +663,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="168">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="3"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
@@ -936,180 +898,32 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="4"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="4"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="4"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="10" fillId="2" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="10" fillId="2" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="3"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="4"/>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="4"/>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="4"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="4"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="23" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="23" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="4"/>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="4"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="4"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1668,7 +1482,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K75"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="16" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.5546875" customWidth="1" style="75" min="1" max="1"/>
     <col width="10.88671875" customWidth="1" style="75" min="2" max="2"/>
@@ -1683,9 +1497,9 @@
     <col width="9.109375" customWidth="1" style="75" min="12" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16" customHeight="1">
+    <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="n"/>
-      <c r="C1" s="98" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>Foresight and Analysis</t>
         </is>
@@ -1693,7 +1507,7 @@
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="C2" s="28" t="inlineStr">
         <is>
@@ -1707,7 +1521,7 @@
       <c r="H2" s="12" t="n"/>
       <c r="I2" s="12" t="n"/>
     </row>
-    <row r="3" ht="16" customHeight="1">
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="n"/>
       <c r="C3" s="12" t="n"/>
       <c r="D3" s="12" t="n"/>
@@ -1717,60 +1531,60 @@
       <c r="H3" s="12" t="n"/>
       <c r="I3" s="12" t="n"/>
     </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="99" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Historical Primary Elevator Storage Capacity, Manitoba</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
     </row>
-    <row r="5" ht="16" customHeight="1" thickBot="1">
+    <row r="5" ht="15" customHeight="1" thickBot="1">
       <c r="A5" s="4" t="n"/>
     </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="100" t="inlineStr">
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B6" s="101" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="C6" s="102" t="inlineStr">
+      <c r="C6" s="98" t="inlineStr">
         <is>
           <t>Total Capacity</t>
         </is>
       </c>
-      <c r="D6" s="103" t="n"/>
-      <c r="E6" s="104" t="inlineStr">
+      <c r="D6" s="99" t="n"/>
+      <c r="E6" s="100" t="inlineStr">
         <is>
           <t>Average Elevator Capacity</t>
         </is>
       </c>
-      <c r="F6" s="105" t="n"/>
-    </row>
-    <row r="7" ht="16" customHeight="1">
+      <c r="F6" s="101" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="16" t="n"/>
       <c r="B7" s="17" t="n"/>
-      <c r="C7" s="106" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>000 tonnes</t>
         </is>
       </c>
-      <c r="D7" s="106" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>000 bushels</t>
         </is>
       </c>
-      <c r="E7" s="106" t="inlineStr">
+      <c r="E7" s="18" t="inlineStr">
         <is>
           <t>000 tonnes</t>
         </is>
       </c>
-      <c r="F7" s="107" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>000 bushels</t>
         </is>
@@ -1781,23 +1595,23 @@
       <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="n"/>
     </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="108" t="n">
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="20" t="n">
         <v>1963</v>
       </c>
-      <c r="B8" s="109" t="n">
+      <c r="B8" s="21" t="n">
         <v>678</v>
       </c>
-      <c r="C8" s="110" t="n">
+      <c r="C8" s="22" t="n">
         <v>1333.2</v>
       </c>
-      <c r="D8" s="109" t="n">
+      <c r="D8" s="21" t="n">
         <v>48985</v>
       </c>
-      <c r="E8" s="110" t="n">
+      <c r="E8" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="111" t="n">
+      <c r="F8" s="23" t="n">
         <v>72.2</v>
       </c>
       <c r="G8" s="9" t="n"/>
@@ -1806,63 +1620,63 @@
       <c r="J8" s="9" t="n"/>
       <c r="K8" s="9" t="n"/>
     </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="112" t="n">
+    <row r="9">
+      <c r="A9" s="24" t="n">
         <v>1964</v>
       </c>
-      <c r="B9" s="113" t="n">
+      <c r="B9" s="25" t="n">
         <v>677</v>
       </c>
-      <c r="C9" s="114" t="n">
+      <c r="C9" s="26" t="n">
         <v>1360.1</v>
       </c>
-      <c r="D9" s="113" t="n">
+      <c r="D9" s="25" t="n">
         <v>49975</v>
       </c>
-      <c r="E9" s="114" t="n">
+      <c r="E9" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="115" t="n">
+      <c r="F9" s="27" t="n">
         <v>73.8</v>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="112" t="n">
+    <row r="10">
+      <c r="A10" s="24" t="n">
         <v>1965</v>
       </c>
-      <c r="B10" s="113" t="n">
+      <c r="B10" s="25" t="n">
         <v>669</v>
       </c>
-      <c r="C10" s="114" t="n">
+      <c r="C10" s="26" t="n">
         <v>1373.6</v>
       </c>
-      <c r="D10" s="113" t="n">
+      <c r="D10" s="25" t="n">
         <v>50470</v>
       </c>
-      <c r="E10" s="114" t="n">
+      <c r="E10" s="26" t="n">
         <v>2.1</v>
       </c>
-      <c r="F10" s="115" t="n">
+      <c r="F10" s="27" t="n">
         <v>75.40000000000001</v>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="112" t="n">
+    <row r="11">
+      <c r="A11" s="24" t="n">
         <v>1966</v>
       </c>
-      <c r="B11" s="113" t="n">
+      <c r="B11" s="25" t="n">
         <v>651</v>
       </c>
-      <c r="C11" s="114" t="n">
+      <c r="C11" s="26" t="n">
         <v>1363.3</v>
       </c>
-      <c r="D11" s="113" t="n">
+      <c r="D11" s="25" t="n">
         <v>50095</v>
       </c>
-      <c r="E11" s="114" t="n">
+      <c r="E11" s="26" t="n">
         <v>2.1</v>
       </c>
-      <c r="F11" s="115" t="n">
+      <c r="F11" s="27" t="n">
         <v>77</v>
       </c>
       <c r="G11" s="6" t="n"/>
@@ -1871,23 +1685,23 @@
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
     </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="112" t="n">
+    <row r="12">
+      <c r="A12" s="24" t="n">
         <v>1967</v>
       </c>
-      <c r="B12" s="113" t="n">
+      <c r="B12" s="25" t="n">
         <v>645</v>
       </c>
-      <c r="C12" s="114" t="n">
+      <c r="C12" s="26" t="n">
         <v>1373.6</v>
       </c>
-      <c r="D12" s="113" t="n">
+      <c r="D12" s="25" t="n">
         <v>50470</v>
       </c>
-      <c r="E12" s="114" t="n">
+      <c r="E12" s="26" t="n">
         <v>2.1</v>
       </c>
-      <c r="F12" s="115" t="n">
+      <c r="F12" s="27" t="n">
         <v>78.2</v>
       </c>
       <c r="G12" s="6" t="n"/>
@@ -1896,23 +1710,23 @@
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
     </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="112" t="n">
+    <row r="13">
+      <c r="A13" s="24" t="n">
         <v>1968</v>
       </c>
-      <c r="B13" s="113" t="n">
+      <c r="B13" s="25" t="n">
         <v>642</v>
       </c>
-      <c r="C13" s="114" t="n">
+      <c r="C13" s="26" t="n">
         <v>1408.1</v>
       </c>
-      <c r="D13" s="113" t="n">
+      <c r="D13" s="25" t="n">
         <v>51740</v>
       </c>
-      <c r="E13" s="114" t="n">
+      <c r="E13" s="26" t="n">
         <v>2.2</v>
       </c>
-      <c r="F13" s="115" t="n">
+      <c r="F13" s="27" t="n">
         <v>80.59999999999999</v>
       </c>
       <c r="G13" s="6" t="n"/>
@@ -1921,23 +1735,23 @@
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
     </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="112" t="n">
+    <row r="14">
+      <c r="A14" s="24" t="n">
         <v>1969</v>
       </c>
-      <c r="B14" s="113" t="n">
+      <c r="B14" s="25" t="n">
         <v>641</v>
       </c>
-      <c r="C14" s="114" t="n">
+      <c r="C14" s="26" t="n">
         <v>1437</v>
       </c>
-      <c r="D14" s="113" t="n">
+      <c r="D14" s="25" t="n">
         <v>52800</v>
       </c>
-      <c r="E14" s="114" t="n">
+      <c r="E14" s="26" t="n">
         <v>2.2</v>
       </c>
-      <c r="F14" s="115" t="n">
+      <c r="F14" s="27" t="n">
         <v>82.40000000000001</v>
       </c>
       <c r="G14" s="6" t="n"/>
@@ -1946,23 +1760,23 @@
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
     </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="112" t="n">
+    <row r="15">
+      <c r="A15" s="24" t="n">
         <v>1970</v>
       </c>
-      <c r="B15" s="113" t="n">
+      <c r="B15" s="25" t="n">
         <v>642</v>
       </c>
-      <c r="C15" s="114" t="n">
+      <c r="C15" s="26" t="n">
         <v>1459</v>
       </c>
-      <c r="D15" s="113" t="n">
+      <c r="D15" s="25" t="n">
         <v>53610</v>
       </c>
-      <c r="E15" s="114" t="n">
+      <c r="E15" s="26" t="n">
         <v>2.3</v>
       </c>
-      <c r="F15" s="115" t="n">
+      <c r="F15" s="27" t="n">
         <v>83.5</v>
       </c>
       <c r="G15" s="6" t="n"/>
@@ -1971,23 +1785,23 @@
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="112" t="n">
+    <row r="16">
+      <c r="A16" s="24" t="n">
         <v>1971</v>
       </c>
-      <c r="B16" s="113" t="n">
+      <c r="B16" s="25" t="n">
         <v>616</v>
       </c>
-      <c r="C16" s="114" t="n">
+      <c r="C16" s="26" t="n">
         <v>1427.7</v>
       </c>
-      <c r="D16" s="113" t="n">
+      <c r="D16" s="25" t="n">
         <v>52460</v>
       </c>
-      <c r="E16" s="114" t="n">
+      <c r="E16" s="26" t="n">
         <v>2.3</v>
       </c>
-      <c r="F16" s="115" t="n">
+      <c r="F16" s="27" t="n">
         <v>85.2</v>
       </c>
       <c r="G16" s="6" t="n"/>
@@ -1996,23 +1810,23 @@
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
     </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="112" t="n">
+    <row r="17">
+      <c r="A17" s="24" t="n">
         <v>1972</v>
       </c>
-      <c r="B17" s="113" t="n">
+      <c r="B17" s="25" t="n">
         <v>574</v>
       </c>
-      <c r="C17" s="114" t="n">
+      <c r="C17" s="26" t="n">
         <v>1348.9</v>
       </c>
-      <c r="D17" s="113" t="n">
+      <c r="D17" s="25" t="n">
         <v>49560</v>
       </c>
-      <c r="E17" s="114" t="n">
+      <c r="E17" s="26" t="n">
         <v>2.3</v>
       </c>
-      <c r="F17" s="115" t="n">
+      <c r="F17" s="27" t="n">
         <v>86.3</v>
       </c>
       <c r="G17" s="6" t="n"/>
@@ -2021,23 +1835,23 @@
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
     </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="112" t="n">
+    <row r="18">
+      <c r="A18" s="24" t="n">
         <v>1973</v>
       </c>
-      <c r="B18" s="113" t="n">
+      <c r="B18" s="25" t="n">
         <v>540</v>
       </c>
-      <c r="C18" s="114" t="n">
+      <c r="C18" s="26" t="n">
         <v>1298.5</v>
       </c>
-      <c r="D18" s="113" t="n">
+      <c r="D18" s="25" t="n">
         <v>47710</v>
       </c>
-      <c r="E18" s="114" t="n">
+      <c r="E18" s="26" t="n">
         <v>2.4</v>
       </c>
-      <c r="F18" s="115" t="n">
+      <c r="F18" s="27" t="n">
         <v>88.40000000000001</v>
       </c>
       <c r="G18" s="6" t="n"/>
@@ -2046,23 +1860,23 @@
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
     </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="112" t="n">
+    <row r="19">
+      <c r="A19" s="24" t="n">
         <v>1974</v>
       </c>
-      <c r="B19" s="113" t="n">
+      <c r="B19" s="25" t="n">
         <v>523</v>
       </c>
-      <c r="C19" s="114" t="n">
+      <c r="C19" s="26" t="n">
         <v>1278.8</v>
       </c>
-      <c r="D19" s="113" t="n">
+      <c r="D19" s="25" t="n">
         <v>46985</v>
       </c>
-      <c r="E19" s="114" t="n">
+      <c r="E19" s="26" t="n">
         <v>2.4</v>
       </c>
-      <c r="F19" s="115" t="n">
+      <c r="F19" s="27" t="n">
         <v>89.8</v>
       </c>
       <c r="G19" s="6" t="n"/>
@@ -2071,23 +1885,23 @@
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="112" t="n">
+    <row r="20">
+      <c r="A20" s="24" t="n">
         <v>1975</v>
       </c>
-      <c r="B20" s="113" t="n">
+      <c r="B20" s="25" t="n">
         <v>502</v>
       </c>
-      <c r="C20" s="114" t="n">
+      <c r="C20" s="26" t="n">
         <v>1257.8</v>
       </c>
-      <c r="D20" s="113" t="n">
+      <c r="D20" s="25" t="n">
         <v>46215</v>
       </c>
-      <c r="E20" s="114" t="n">
+      <c r="E20" s="26" t="n">
         <v>2.5</v>
       </c>
-      <c r="F20" s="115" t="n">
+      <c r="F20" s="27" t="n">
         <v>92.09999999999999</v>
       </c>
       <c r="G20" s="6" t="n"/>
@@ -2096,23 +1910,23 @@
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="6" t="n"/>
     </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="112" t="n">
+    <row r="21">
+      <c r="A21" s="24" t="n">
         <v>1976</v>
       </c>
-      <c r="B21" s="113" t="n">
+      <c r="B21" s="25" t="n">
         <v>480</v>
       </c>
-      <c r="C21" s="114" t="n">
+      <c r="C21" s="26" t="n">
         <v>1239.2</v>
       </c>
-      <c r="D21" s="113" t="n">
+      <c r="D21" s="25" t="n">
         <v>45535</v>
       </c>
-      <c r="E21" s="114" t="n">
+      <c r="E21" s="26" t="n">
         <v>2.6</v>
       </c>
-      <c r="F21" s="115" t="n">
+      <c r="F21" s="27" t="n">
         <v>94.90000000000001</v>
       </c>
       <c r="G21" s="6" t="n"/>
@@ -2121,23 +1935,23 @@
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
     </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="112" t="n">
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="24" t="n">
         <v>1977</v>
       </c>
-      <c r="B22" s="113" t="n">
+      <c r="B22" s="25" t="n">
         <v>454</v>
       </c>
-      <c r="C22" s="114" t="n">
+      <c r="C22" s="26" t="n">
         <v>1206.6</v>
       </c>
-      <c r="D22" s="113" t="n">
+      <c r="D22" s="25" t="n">
         <v>44335</v>
       </c>
-      <c r="E22" s="114" t="n">
+      <c r="E22" s="26" t="n">
         <v>2.7</v>
       </c>
-      <c r="F22" s="115" t="n">
+      <c r="F22" s="27" t="n">
         <v>97.7</v>
       </c>
       <c r="G22" s="8" t="n"/>
@@ -2146,83 +1960,83 @@
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
     </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="112" t="n">
+    <row r="23">
+      <c r="A23" s="24" t="n">
         <v>1978</v>
       </c>
-      <c r="B23" s="113" t="n">
+      <c r="B23" s="25" t="n">
         <v>446</v>
       </c>
-      <c r="C23" s="114" t="n">
+      <c r="C23" s="26" t="n">
         <v>1216.4</v>
       </c>
-      <c r="D23" s="113" t="n">
+      <c r="D23" s="25" t="n">
         <v>44695</v>
       </c>
-      <c r="E23" s="114" t="n">
+      <c r="E23" s="26" t="n">
         <v>2.7</v>
       </c>
-      <c r="F23" s="115" t="n">
+      <c r="F23" s="27" t="n">
         <v>100.2</v>
       </c>
     </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="112" t="n">
+    <row r="24">
+      <c r="A24" s="24" t="n">
         <v>1979</v>
       </c>
-      <c r="B24" s="113" t="n">
+      <c r="B24" s="25" t="n">
         <v>417</v>
       </c>
-      <c r="C24" s="114" t="n">
+      <c r="C24" s="26" t="n">
         <v>1177.2</v>
       </c>
-      <c r="D24" s="113" t="n">
+      <c r="D24" s="25" t="n">
         <v>43255</v>
       </c>
-      <c r="E24" s="114" t="n">
+      <c r="E24" s="26" t="n">
         <v>2.8</v>
       </c>
-      <c r="F24" s="115" t="n">
+      <c r="F24" s="27" t="n">
         <v>103.7</v>
       </c>
     </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="112" t="n">
+    <row r="25">
+      <c r="A25" s="24" t="n">
         <v>1980</v>
       </c>
-      <c r="B25" s="113" t="n">
+      <c r="B25" s="25" t="n">
         <v>405</v>
       </c>
-      <c r="C25" s="114" t="n">
+      <c r="C25" s="26" t="n">
         <v>1173.1</v>
       </c>
-      <c r="D25" s="113" t="n">
+      <c r="D25" s="25" t="n">
         <v>43105</v>
       </c>
-      <c r="E25" s="114" t="n">
+      <c r="E25" s="26" t="n">
         <v>2.9</v>
       </c>
-      <c r="F25" s="115" t="n">
+      <c r="F25" s="27" t="n">
         <v>106.4</v>
       </c>
     </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="112" t="n">
+    <row r="26">
+      <c r="A26" s="24" t="n">
         <v>1981</v>
       </c>
-      <c r="B26" s="113" t="n">
+      <c r="B26" s="25" t="n">
         <v>373</v>
       </c>
-      <c r="C26" s="114" t="n">
+      <c r="C26" s="26" t="n">
         <v>1135.5</v>
       </c>
-      <c r="D26" s="113" t="n">
+      <c r="D26" s="25" t="n">
         <v>41720</v>
       </c>
-      <c r="E26" s="114" t="n">
+      <c r="E26" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="F26" s="115" t="n">
+      <c r="F26" s="27" t="n">
         <v>111.8</v>
       </c>
       <c r="G26" s="10" t="n"/>
@@ -2231,928 +2045,927 @@
       <c r="J26" s="10" t="n"/>
       <c r="K26" s="10" t="n"/>
     </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="112" t="n">
+    <row r="27">
+      <c r="A27" s="24" t="n">
         <v>1982</v>
       </c>
-      <c r="B27" s="113" t="n">
+      <c r="B27" s="25" t="n">
         <v>361</v>
       </c>
-      <c r="C27" s="114" t="n">
+      <c r="C27" s="26" t="n">
         <v>1142.6</v>
       </c>
-      <c r="D27" s="113" t="n">
+      <c r="D27" s="25" t="n">
         <v>41980</v>
       </c>
-      <c r="E27" s="114" t="n">
+      <c r="E27" s="26" t="n">
         <v>3.2</v>
       </c>
-      <c r="F27" s="115" t="n">
+      <c r="F27" s="27" t="n">
         <v>116.3</v>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="112" t="n">
+    <row r="28">
+      <c r="A28" s="24" t="n">
         <v>1983</v>
       </c>
-      <c r="B28" s="113" t="n">
+      <c r="B28" s="25" t="n">
         <v>364</v>
       </c>
-      <c r="C28" s="114" t="n">
+      <c r="C28" s="26" t="n">
         <v>1157.4</v>
       </c>
-      <c r="D28" s="113" t="n">
+      <c r="D28" s="25" t="n">
         <v>42530</v>
       </c>
-      <c r="E28" s="114" t="n">
+      <c r="E28" s="26" t="n">
         <v>3.2</v>
       </c>
-      <c r="F28" s="115" t="n">
+      <c r="F28" s="27" t="n">
         <v>116.8</v>
       </c>
     </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="112" t="n">
+    <row r="29">
+      <c r="A29" s="24" t="n">
         <v>1984</v>
       </c>
-      <c r="B29" s="113" t="n">
+      <c r="B29" s="25" t="n">
         <v>309</v>
       </c>
-      <c r="C29" s="114" t="n">
+      <c r="C29" s="26" t="n">
         <v>1131</v>
       </c>
-      <c r="D29" s="113" t="n">
+      <c r="D29" s="25" t="n">
         <v>41555</v>
       </c>
-      <c r="E29" s="114" t="n">
+      <c r="E29" s="26" t="n">
         <v>3.7</v>
       </c>
-      <c r="F29" s="115" t="n">
+      <c r="F29" s="27" t="n">
         <v>134.5</v>
       </c>
     </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="112" t="n">
+    <row r="30">
+      <c r="A30" s="24" t="n">
         <v>1985</v>
       </c>
-      <c r="B30" s="113" t="n">
+      <c r="B30" s="25" t="n">
         <v>305</v>
       </c>
-      <c r="C30" s="114" t="n">
+      <c r="C30" s="26" t="n">
         <v>1124.5</v>
       </c>
-      <c r="D30" s="113" t="n">
+      <c r="D30" s="25" t="n">
         <v>41320</v>
       </c>
-      <c r="E30" s="114" t="n">
+      <c r="E30" s="26" t="n">
         <v>3.7</v>
       </c>
-      <c r="F30" s="115" t="n">
+      <c r="F30" s="27" t="n">
         <v>135.5</v>
       </c>
     </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="112" t="n">
+    <row r="31">
+      <c r="A31" s="24" t="n">
         <v>1986</v>
       </c>
-      <c r="B31" s="113" t="n">
+      <c r="B31" s="25" t="n">
         <v>292</v>
       </c>
-      <c r="C31" s="114" t="n">
+      <c r="C31" s="26" t="n">
         <v>1114.8</v>
       </c>
-      <c r="D31" s="113" t="n">
+      <c r="D31" s="25" t="n">
         <v>40965</v>
       </c>
-      <c r="E31" s="114" t="n">
+      <c r="E31" s="26" t="n">
         <v>3.8</v>
       </c>
-      <c r="F31" s="115" t="n">
+      <c r="F31" s="27" t="n">
         <v>140.3</v>
       </c>
     </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="112" t="n">
+    <row r="32">
+      <c r="A32" s="24" t="n">
         <v>1987</v>
       </c>
-      <c r="B32" s="113" t="n">
+      <c r="B32" s="25" t="n">
         <v>288</v>
       </c>
-      <c r="C32" s="114" t="n">
+      <c r="C32" s="26" t="n">
         <v>1106.3</v>
       </c>
-      <c r="D32" s="113" t="n">
+      <c r="D32" s="25" t="n">
         <v>40650</v>
       </c>
-      <c r="E32" s="114" t="n">
+      <c r="E32" s="26" t="n">
         <v>3.8</v>
       </c>
-      <c r="F32" s="115" t="n">
+      <c r="F32" s="27" t="n">
         <v>141.1</v>
       </c>
     </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="112" t="n">
+    <row r="33">
+      <c r="A33" s="24" t="n">
         <v>1988</v>
       </c>
-      <c r="B33" s="113" t="n">
+      <c r="B33" s="25" t="n">
         <v>284</v>
       </c>
-      <c r="C33" s="114" t="n">
+      <c r="C33" s="26" t="n">
         <v>1104.5</v>
       </c>
-      <c r="D33" s="113" t="n">
+      <c r="D33" s="25" t="n">
         <v>40580</v>
       </c>
-      <c r="E33" s="114" t="n">
+      <c r="E33" s="26" t="n">
         <v>3.9</v>
       </c>
-      <c r="F33" s="115" t="n">
+      <c r="F33" s="27" t="n">
         <v>142.9</v>
       </c>
     </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="112" t="n">
+    <row r="34">
+      <c r="A34" s="24" t="n">
         <v>1989</v>
       </c>
-      <c r="B34" s="113" t="n">
+      <c r="B34" s="25" t="n">
         <v>272</v>
       </c>
-      <c r="C34" s="114" t="n">
+      <c r="C34" s="26" t="n">
         <v>1071.9</v>
       </c>
-      <c r="D34" s="113" t="n">
+      <c r="D34" s="25" t="n">
         <v>39385</v>
       </c>
-      <c r="E34" s="114" t="n">
+      <c r="E34" s="26" t="n">
         <v>3.9</v>
       </c>
-      <c r="F34" s="115" t="n">
+      <c r="F34" s="27" t="n">
         <v>144.8</v>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="112" t="n">
+    <row r="35">
+      <c r="A35" s="24" t="n">
         <v>1990</v>
       </c>
-      <c r="B35" s="113" t="n">
+      <c r="B35" s="25" t="n">
         <v>264</v>
       </c>
-      <c r="C35" s="114" t="n">
+      <c r="C35" s="26" t="n">
         <v>1110.1</v>
       </c>
-      <c r="D35" s="113" t="n">
+      <c r="D35" s="25" t="n">
         <v>40790</v>
       </c>
-      <c r="E35" s="114" t="n">
+      <c r="E35" s="26" t="n">
         <v>4.2</v>
       </c>
-      <c r="F35" s="115" t="n">
+      <c r="F35" s="27" t="n">
         <v>154.5</v>
       </c>
     </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="112" t="n">
+    <row r="36">
+      <c r="A36" s="24" t="n">
         <v>1991</v>
       </c>
-      <c r="B36" s="113" t="n">
+      <c r="B36" s="25" t="n">
         <v>258</v>
       </c>
-      <c r="C36" s="114" t="n">
+      <c r="C36" s="26" t="n">
         <v>1094.1</v>
       </c>
-      <c r="D36" s="113" t="n">
+      <c r="D36" s="25" t="n">
         <v>40200</v>
       </c>
-      <c r="E36" s="114" t="n">
+      <c r="E36" s="26" t="n">
         <v>4.2</v>
       </c>
-      <c r="F36" s="115" t="n">
+      <c r="F36" s="27" t="n">
         <v>155.8</v>
       </c>
     </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="112" t="n">
+    <row r="37">
+      <c r="A37" s="24" t="n">
         <v>1992</v>
       </c>
-      <c r="B37" s="113" t="n">
+      <c r="B37" s="25" t="n">
         <v>256</v>
       </c>
-      <c r="C37" s="114" t="n">
+      <c r="C37" s="26" t="n">
         <v>1086.5</v>
       </c>
-      <c r="D37" s="113" t="n">
+      <c r="D37" s="25" t="n">
         <v>39920</v>
       </c>
-      <c r="E37" s="114" t="n">
+      <c r="E37" s="26" t="n">
         <v>4.2</v>
       </c>
-      <c r="F37" s="115" t="n">
+      <c r="F37" s="27" t="n">
         <v>155.9</v>
       </c>
     </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="112" t="n">
+    <row r="38">
+      <c r="A38" s="24" t="n">
         <v>1993</v>
       </c>
-      <c r="B38" s="113" t="n">
+      <c r="B38" s="25" t="n">
         <v>254</v>
       </c>
-      <c r="C38" s="114" t="n">
+      <c r="C38" s="26" t="n">
         <v>1083.7</v>
       </c>
-      <c r="D38" s="113" t="n">
+      <c r="D38" s="25" t="n">
         <v>39820</v>
       </c>
-      <c r="E38" s="114" t="n">
+      <c r="E38" s="26" t="n">
         <v>4.3</v>
       </c>
-      <c r="F38" s="115" t="n">
+      <c r="F38" s="27" t="n">
         <v>156.8</v>
       </c>
     </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="112" t="n">
+    <row r="39">
+      <c r="A39" s="24" t="n">
         <v>1994</v>
       </c>
-      <c r="B39" s="113" t="n">
+      <c r="B39" s="25" t="n">
         <v>251</v>
       </c>
-      <c r="C39" s="114" t="n">
+      <c r="C39" s="26" t="n">
         <v>1072.4</v>
       </c>
-      <c r="D39" s="113" t="n">
+      <c r="D39" s="25" t="n">
         <v>39405</v>
       </c>
-      <c r="E39" s="114" t="n">
+      <c r="E39" s="26" t="n">
         <v>4.3</v>
       </c>
-      <c r="F39" s="115" t="n">
+      <c r="F39" s="27" t="n">
         <v>157</v>
       </c>
     </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="112" t="n">
+    <row r="40">
+      <c r="A40" s="24" t="n">
         <v>1995</v>
       </c>
-      <c r="B40" s="113" t="n">
+      <c r="B40" s="25" t="n">
         <v>236</v>
       </c>
-      <c r="C40" s="114" t="n">
+      <c r="C40" s="26" t="n">
         <v>1072.8</v>
       </c>
-      <c r="D40" s="113" t="n">
+      <c r="D40" s="25" t="n">
         <v>39420</v>
       </c>
-      <c r="E40" s="114" t="n">
+      <c r="E40" s="26" t="n">
         <v>4.5</v>
       </c>
-      <c r="F40" s="115" t="n">
+      <c r="F40" s="27" t="n">
         <v>167</v>
       </c>
     </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="112" t="n">
+    <row r="41">
+      <c r="A41" s="24" t="n">
         <v>1996</v>
       </c>
-      <c r="B41" s="113" t="n">
+      <c r="B41" s="25" t="n">
         <v>220</v>
       </c>
-      <c r="C41" s="114" t="n">
+      <c r="C41" s="26" t="n">
         <v>1040.3</v>
       </c>
-      <c r="D41" s="113" t="n">
+      <c r="D41" s="25" t="n">
         <v>38225</v>
       </c>
-      <c r="E41" s="114" t="n">
+      <c r="E41" s="26" t="n">
         <v>4.7</v>
       </c>
-      <c r="F41" s="115" t="n">
+      <c r="F41" s="27" t="n">
         <v>173.8</v>
       </c>
     </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="112" t="n">
+    <row r="42">
+      <c r="A42" s="24" t="n">
         <v>1997</v>
       </c>
-      <c r="B42" s="113" t="n">
+      <c r="B42" s="25" t="n">
         <v>212</v>
       </c>
-      <c r="C42" s="114" t="n">
+      <c r="C42" s="26" t="n">
         <v>1016.6</v>
       </c>
-      <c r="D42" s="113" t="n">
+      <c r="D42" s="25" t="n">
         <v>37355</v>
       </c>
-      <c r="E42" s="114" t="n">
+      <c r="E42" s="26" t="n">
         <v>4.8</v>
       </c>
-      <c r="F42" s="115" t="n">
+      <c r="F42" s="27" t="n">
         <v>176.2</v>
       </c>
     </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="112" t="n">
+    <row r="43">
+      <c r="A43" s="24" t="n">
         <v>1998</v>
       </c>
-      <c r="B43" s="113" t="n">
+      <c r="B43" s="25" t="n">
         <v>209</v>
       </c>
-      <c r="C43" s="114" t="n">
+      <c r="C43" s="26" t="n">
         <v>1063.6</v>
       </c>
-      <c r="D43" s="113" t="n">
+      <c r="D43" s="25" t="n">
         <v>39080</v>
       </c>
-      <c r="E43" s="114" t="n">
+      <c r="E43" s="26" t="n">
         <v>5.1</v>
       </c>
-      <c r="F43" s="115" t="n">
+      <c r="F43" s="27" t="n">
         <v>187</v>
       </c>
     </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="112" t="n">
+    <row r="44">
+      <c r="A44" s="24" t="n">
         <v>1999</v>
       </c>
-      <c r="B44" s="113" t="n">
+      <c r="B44" s="25" t="n">
         <v>208</v>
       </c>
-      <c r="C44" s="114" t="n">
+      <c r="C44" s="26" t="n">
         <v>1168.5</v>
       </c>
-      <c r="D44" s="113" t="n">
+      <c r="D44" s="25" t="n">
         <v>42935</v>
       </c>
-      <c r="E44" s="114" t="n">
+      <c r="E44" s="26" t="n">
         <v>5.6</v>
       </c>
-      <c r="F44" s="115" t="n">
+      <c r="F44" s="27" t="n">
         <v>206.4</v>
       </c>
     </row>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="112" t="n">
+    <row r="45">
+      <c r="A45" s="24" t="n">
         <v>2000</v>
       </c>
-      <c r="B45" s="113" t="n">
+      <c r="B45" s="25" t="n">
         <v>196</v>
       </c>
-      <c r="C45" s="114" t="n">
+      <c r="C45" s="26" t="n">
         <v>1251.1</v>
       </c>
-      <c r="D45" s="113" t="n">
+      <c r="D45" s="25" t="n">
         <v>45970</v>
       </c>
-      <c r="E45" s="114" t="n">
+      <c r="E45" s="26" t="n">
         <v>6.4</v>
       </c>
-      <c r="F45" s="115" t="n">
+      <c r="F45" s="27" t="n">
         <v>234.5</v>
       </c>
     </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="112" t="n">
+    <row r="46">
+      <c r="A46" s="24" t="n">
         <v>2001</v>
       </c>
-      <c r="B46" s="113" t="n">
+      <c r="B46" s="25" t="n">
         <v>165</v>
       </c>
-      <c r="C46" s="114" t="n">
+      <c r="C46" s="26" t="n">
         <v>1240.1</v>
       </c>
-      <c r="D46" s="113" t="n">
+      <c r="D46" s="25" t="n">
         <v>45565</v>
       </c>
-      <c r="E46" s="114" t="n">
+      <c r="E46" s="26" t="n">
         <v>7.5</v>
       </c>
-      <c r="F46" s="115" t="n">
+      <c r="F46" s="27" t="n">
         <v>276.2</v>
       </c>
     </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="112" t="n">
+    <row r="47">
+      <c r="A47" s="24" t="n">
         <v>2002</v>
       </c>
-      <c r="B47" s="113" t="n">
+      <c r="B47" s="25" t="n">
         <v>100</v>
       </c>
-      <c r="C47" s="114" t="n">
+      <c r="C47" s="26" t="n">
         <v>992.2</v>
       </c>
-      <c r="D47" s="113" t="n">
+      <c r="D47" s="25" t="n">
         <v>36455</v>
       </c>
-      <c r="E47" s="114" t="n">
+      <c r="E47" s="26" t="n">
         <v>9.9</v>
       </c>
-      <c r="F47" s="115" t="n">
+      <c r="F47" s="27" t="n">
         <v>364.6</v>
       </c>
     </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="112" t="n">
+    <row r="48">
+      <c r="A48" s="24" t="n">
         <v>2003</v>
       </c>
-      <c r="B48" s="113" t="n">
+      <c r="B48" s="25" t="n">
         <v>90</v>
       </c>
-      <c r="C48" s="114" t="n">
+      <c r="C48" s="26" t="n">
         <v>963.1</v>
       </c>
-      <c r="D48" s="113" t="n">
+      <c r="D48" s="25" t="n">
         <v>35390</v>
       </c>
-      <c r="E48" s="114" t="n">
+      <c r="E48" s="26" t="n">
         <v>10.7</v>
       </c>
-      <c r="F48" s="115" t="n">
+      <c r="F48" s="27" t="n">
         <v>393.2</v>
       </c>
     </row>
-    <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="112" t="n">
+    <row r="49">
+      <c r="A49" s="24" t="n">
         <v>2004</v>
       </c>
-      <c r="B49" s="113" t="n">
+      <c r="B49" s="25" t="n">
         <v>78</v>
       </c>
-      <c r="C49" s="114" t="n">
+      <c r="C49" s="26" t="n">
         <v>923.4</v>
       </c>
-      <c r="D49" s="113" t="n">
+      <c r="D49" s="25" t="n">
         <v>33930</v>
       </c>
-      <c r="E49" s="114" t="n">
+      <c r="E49" s="26" t="n">
         <v>11.8</v>
       </c>
-      <c r="F49" s="115" t="n">
+      <c r="F49" s="27" t="n">
         <v>433.6</v>
       </c>
     </row>
-    <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="112" t="n">
+    <row r="50">
+      <c r="A50" s="24" t="n">
         <v>2005</v>
       </c>
-      <c r="B50" s="113" t="n">
+      <c r="B50" s="25" t="n">
         <v>75</v>
       </c>
-      <c r="C50" s="114" t="n">
+      <c r="C50" s="26" t="n">
         <v>941.1</v>
       </c>
-      <c r="D50" s="113" t="n">
+      <c r="D50" s="25" t="n">
         <v>34580</v>
       </c>
-      <c r="E50" s="114" t="n">
+      <c r="E50" s="26" t="n">
         <v>12.5</v>
       </c>
-      <c r="F50" s="115" t="n">
+      <c r="F50" s="27" t="n">
         <v>459.3</v>
       </c>
     </row>
-    <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="112" t="n">
+    <row r="51">
+      <c r="A51" s="24" t="n">
         <v>2006</v>
       </c>
-      <c r="B51" s="113" t="n">
+      <c r="B51" s="25" t="n">
         <v>72</v>
       </c>
-      <c r="C51" s="114" t="n">
+      <c r="C51" s="26" t="n">
         <v>918.2</v>
       </c>
-      <c r="D51" s="113" t="n">
+      <c r="D51" s="25" t="n">
         <v>33739</v>
       </c>
-      <c r="E51" s="114" t="n">
+      <c r="E51" s="26" t="n">
         <v>12.8</v>
       </c>
-      <c r="F51" s="115" t="n">
+      <c r="F51" s="27" t="n">
         <v>468.6</v>
       </c>
     </row>
-    <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="112" t="n">
+    <row r="52">
+      <c r="A52" s="24" t="n">
         <v>2007</v>
       </c>
-      <c r="B52" s="113" t="n">
+      <c r="B52" s="25" t="n">
         <v>75</v>
       </c>
-      <c r="C52" s="114" t="n">
+      <c r="C52" s="26" t="n">
         <v>936.7</v>
       </c>
-      <c r="D52" s="113" t="n">
+      <c r="D52" s="25" t="n">
         <v>34417</v>
       </c>
-      <c r="E52" s="114" t="n">
+      <c r="E52" s="26" t="n">
         <v>12.5</v>
       </c>
-      <c r="F52" s="115" t="n">
+      <c r="F52" s="27" t="n">
         <v>458.9</v>
       </c>
     </row>
-    <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="112" t="n">
+    <row r="53">
+      <c r="A53" s="24" t="n">
         <v>2008</v>
       </c>
-      <c r="B53" s="113" t="n">
+      <c r="B53" s="25" t="n">
         <v>74</v>
       </c>
-      <c r="C53" s="114" t="n">
+      <c r="C53" s="26" t="n">
         <v>1001</v>
       </c>
-      <c r="D53" s="113" t="n">
+      <c r="D53" s="25" t="n">
         <v>36776</v>
       </c>
-      <c r="E53" s="114" t="n">
+      <c r="E53" s="26" t="n">
         <v>13.5</v>
       </c>
-      <c r="F53" s="115" t="n">
+      <c r="F53" s="27" t="n">
         <v>497</v>
       </c>
     </row>
-    <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="112" t="n">
+    <row r="54">
+      <c r="A54" s="24" t="n">
         <v>2009</v>
       </c>
-      <c r="B54" s="113" t="n">
+      <c r="B54" s="25" t="n">
         <v>73</v>
       </c>
-      <c r="C54" s="114" t="n">
+      <c r="C54" s="26" t="n">
         <v>1005.61</v>
       </c>
-      <c r="D54" s="113" t="n">
+      <c r="D54" s="25" t="n">
         <v>36950.13384</v>
       </c>
-      <c r="E54" s="114" t="n">
+      <c r="E54" s="26" t="n">
         <v>13.77547945205479</v>
       </c>
-      <c r="F54" s="115" t="n">
+      <c r="F54" s="27" t="n">
         <v>506.1662169863014</v>
       </c>
     </row>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="112" t="n">
+    <row r="55">
+      <c r="A55" s="24" t="n">
         <v>2010</v>
       </c>
-      <c r="B55" s="113" t="n">
+      <c r="B55" s="25" t="n">
         <v>77</v>
       </c>
-      <c r="C55" s="114" t="n">
+      <c r="C55" s="26" t="n">
         <v>1054.58</v>
       </c>
-      <c r="D55" s="113" t="n">
+      <c r="D55" s="25" t="n">
         <v>38749.48752</v>
       </c>
-      <c r="E55" s="114" t="n">
+      <c r="E55" s="26" t="n">
         <v>13.69584415584415</v>
       </c>
-      <c r="F55" s="115" t="n">
+      <c r="F55" s="27" t="n">
         <v>503.2400976623376</v>
       </c>
     </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="112" t="n">
+    <row r="56">
+      <c r="A56" s="24" t="n">
         <v>2011</v>
       </c>
-      <c r="B56" s="113" t="n">
+      <c r="B56" s="25" t="n">
         <v>85</v>
       </c>
-      <c r="C56" s="114" t="n">
+      <c r="C56" s="26" t="n">
         <v>1285.56</v>
       </c>
-      <c r="D56" s="113" t="n">
+      <c r="D56" s="25" t="n">
         <v>47236.61664</v>
       </c>
-      <c r="E56" s="114" t="n">
+      <c r="E56" s="26" t="n">
         <v>15.12423529411765</v>
       </c>
-      <c r="F56" s="115" t="n">
+      <c r="F56" s="27" t="n">
         <v>555.7249016470588</v>
       </c>
     </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="112" t="n">
+    <row r="57">
+      <c r="A57" s="24" t="n">
         <v>2012</v>
       </c>
-      <c r="B57" s="113" t="n">
+      <c r="B57" s="25" t="n">
         <v>86</v>
       </c>
-      <c r="C57" s="114" t="n">
+      <c r="C57" s="26" t="n">
         <v>1174.88</v>
       </c>
-      <c r="D57" s="113" t="n">
+      <c r="D57" s="25" t="n">
         <v>43169.79072</v>
       </c>
-      <c r="E57" s="114" t="n">
+      <c r="E57" s="26" t="n">
         <v>13.66139534883721</v>
       </c>
-      <c r="F57" s="115" t="n">
+      <c r="F57" s="27" t="n">
         <v>502.369614</v>
       </c>
     </row>
-    <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="112" t="n">
+    <row r="58">
+      <c r="A58" s="24" t="n">
         <v>2013</v>
       </c>
-      <c r="B58" s="113" t="n">
+      <c r="B58" s="25" t="n">
         <v>89</v>
       </c>
-      <c r="C58" s="114" t="n">
+      <c r="C58" s="26" t="n">
         <v>1188.28</v>
       </c>
-      <c r="D58" s="113" t="n">
+      <c r="D58" s="25" t="n">
         <v>43662.16032</v>
       </c>
-      <c r="E58" s="114" t="n">
+      <c r="E58" s="26" t="n">
         <v>13.3514606741573</v>
       </c>
-      <c r="F58" s="115" t="n">
+      <c r="F58" s="27" t="n">
         <v>490.5860710112359</v>
       </c>
     </row>
-    <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="112" t="n">
+    <row r="59">
+      <c r="A59" s="24" t="n">
         <v>2014</v>
       </c>
-      <c r="B59" s="113" t="n">
+      <c r="B59" s="25" t="n">
         <v>82</v>
       </c>
-      <c r="C59" s="114" t="n">
+      <c r="C59" s="26" t="n">
         <v>1344.49</v>
       </c>
-      <c r="D59" s="113" t="n">
+      <c r="D59" s="25" t="n">
         <v>49401.94056</v>
       </c>
-      <c r="E59" s="114" t="n">
+      <c r="E59" s="26" t="n">
         <v>16.39621951219512</v>
       </c>
-      <c r="F59" s="115" t="n">
+      <c r="F59" s="27" t="n">
         <v>602.4626897560976</v>
       </c>
     </row>
-    <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="112" t="n">
+    <row r="60">
+      <c r="A60" s="24" t="n">
         <v>2015</v>
       </c>
-      <c r="B60" s="113" t="n">
+      <c r="B60" s="25" t="n">
         <v>80</v>
       </c>
-      <c r="C60" s="114" t="n">
+      <c r="C60" s="26" t="n">
         <v>1300.06</v>
       </c>
-      <c r="D60" s="113" t="n">
+      <c r="D60" s="25" t="n">
         <v>47769.40464</v>
       </c>
-      <c r="E60" s="114" t="n">
+      <c r="E60" s="26" t="n">
         <v>16.25075</v>
       </c>
-      <c r="F60" s="115" t="n">
+      <c r="F60" s="27" t="n">
         <v>597.117558</v>
       </c>
     </row>
-    <row r="61" ht="16" customHeight="1">
-      <c r="A61" s="112" t="n">
+    <row r="61">
+      <c r="A61" s="24" t="n">
         <v>2016</v>
       </c>
-      <c r="B61" s="113" t="n">
+      <c r="B61" s="25" t="n">
         <v>82</v>
       </c>
-      <c r="C61" s="114" t="n">
+      <c r="C61" s="26" t="n">
         <v>1496.11</v>
       </c>
-      <c r="D61" s="113" t="n">
+      <c r="D61" s="25" t="n">
         <v>54973.06584</v>
       </c>
-      <c r="E61" s="114" t="n">
+      <c r="E61" s="26" t="n">
         <v>18.24524390243903</v>
       </c>
-      <c r="F61" s="115" t="n">
+      <c r="F61" s="27" t="n">
         <v>670.4032419512196</v>
       </c>
     </row>
-    <row r="62" ht="16" customHeight="1">
-      <c r="A62" s="112" t="n">
+    <row r="62">
+      <c r="A62" s="24" t="n">
         <v>2017</v>
       </c>
-      <c r="B62" s="113" t="n">
+      <c r="B62" s="25" t="n">
         <v>84</v>
       </c>
-      <c r="C62" s="114" t="n">
+      <c r="C62" s="26" t="n">
         <v>1594.48</v>
       </c>
-      <c r="D62" s="113" t="n">
+      <c r="D62" s="25" t="n">
         <v>58587.57312</v>
       </c>
-      <c r="E62" s="114" t="n">
+      <c r="E62" s="26" t="n">
         <v>18.9819047619048</v>
       </c>
-      <c r="F62" s="115" t="n">
+      <c r="F62" s="27" t="n">
         <v>697.471108571429</v>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="A63" s="112" t="n">
+    <row r="63">
+      <c r="A63" s="24" t="n">
         <v>2018</v>
       </c>
-      <c r="B63" s="113" t="n">
+      <c r="B63" s="25" t="n">
         <v>84</v>
       </c>
-      <c r="C63" s="114" t="n">
+      <c r="C63" s="26" t="n">
         <v>1598.274</v>
       </c>
-      <c r="D63" s="113" t="n">
+      <c r="D63" s="25" t="n">
         <v>58727.9</v>
       </c>
-      <c r="E63" s="114" t="n">
+      <c r="E63" s="26" t="n">
         <v>19.0270714285714</v>
       </c>
-      <c r="F63" s="115" t="n">
+      <c r="F63" s="27" t="n">
         <v>699.1</v>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="116" t="n">
+    <row r="64">
+      <c r="A64" s="29" t="n">
         <v>2019</v>
       </c>
-      <c r="B64" s="117" t="n">
+      <c r="B64" s="34" t="n">
         <v>85</v>
       </c>
-      <c r="C64" s="118" t="n">
+      <c r="C64" s="30" t="n">
         <v>1615.7</v>
       </c>
-      <c r="D64" s="119" t="n">
+      <c r="D64" s="31" t="n">
         <v>59367.2808</v>
       </c>
-      <c r="E64" s="120" t="n">
+      <c r="E64" s="32" t="n">
         <v>19.00823529411765</v>
       </c>
-      <c r="F64" s="121" t="n">
+      <c r="F64" s="33" t="n">
         <v>698.4385976470588</v>
       </c>
     </row>
-    <row r="65" ht="16" customHeight="1">
-      <c r="A65" s="116" t="n">
+    <row r="65">
+      <c r="A65" s="29" t="n">
         <v>2020</v>
       </c>
-      <c r="B65" s="122" t="n">
+      <c r="B65" s="65" t="n">
         <v>83</v>
       </c>
-      <c r="C65" s="118" t="n">
+      <c r="C65" s="30" t="n">
         <v>1620.6</v>
       </c>
-      <c r="D65" s="119" t="n">
+      <c r="D65" s="31" t="n">
         <v>59547.3264</v>
       </c>
-      <c r="E65" s="120" t="n">
+      <c r="E65" s="32" t="n">
         <v>19.52530120481928</v>
       </c>
-      <c r="F65" s="121" t="n">
+      <c r="F65" s="33" t="n">
         <v>717.4376674698794</v>
       </c>
     </row>
-    <row r="66" ht="16" customHeight="1">
-      <c r="A66" s="116" t="n">
+    <row r="66">
+      <c r="A66" s="29" t="n">
         <v>2021</v>
       </c>
-      <c r="B66" s="122" t="n">
+      <c r="B66" s="65" t="n">
         <v>80</v>
       </c>
-      <c r="C66" s="118" t="n">
+      <c r="C66" s="30" t="n">
         <v>1621.8</v>
       </c>
-      <c r="D66" s="123" t="n">
+      <c r="D66" s="73" t="n">
         <v>59591.4192</v>
       </c>
-      <c r="E66" s="120" t="n">
+      <c r="E66" s="32" t="n">
         <v>20.2725</v>
       </c>
-      <c r="F66" s="121" t="n">
+      <c r="F66" s="33" t="n">
         <v>744.89274</v>
       </c>
     </row>
-    <row r="67" ht="16" customHeight="1">
-      <c r="A67" s="116" t="n">
+    <row r="67">
+      <c r="A67" s="29" t="n">
         <v>2022</v>
       </c>
-      <c r="B67" s="122" t="n">
+      <c r="B67" s="65" t="n">
         <v>83</v>
       </c>
-      <c r="C67" s="118" t="n">
+      <c r="C67" s="30" t="n">
         <v>1682</v>
       </c>
-      <c r="D67" s="123" t="n">
+      <c r="D67" s="73" t="n">
         <v>61802.9034</v>
       </c>
-      <c r="E67" s="120" t="n">
+      <c r="E67" s="32" t="n">
         <v>20.26506024096386</v>
       </c>
-      <c r="F67" s="121" t="n">
+      <c r="F67" s="33" t="n">
         <v>744.6132939759035</v>
       </c>
     </row>
-    <row r="68" ht="16" customHeight="1">
-      <c r="A68" s="116" t="n">
+    <row r="68">
+      <c r="A68" s="29" t="n">
         <v>2023</v>
       </c>
-      <c r="B68" s="122" t="n">
+      <c r="B68" s="65" t="n">
         <v>81</v>
       </c>
-      <c r="C68" s="118" t="n">
+      <c r="C68" s="30" t="n">
         <v>1683.74</v>
       </c>
-      <c r="D68" s="123" t="n">
+      <c r="D68" s="73" t="n">
         <v>61866.837438</v>
       </c>
-      <c r="E68" s="120" t="n">
+      <c r="E68" s="32" t="n">
         <v>20.78691358024691</v>
       </c>
-      <c r="F68" s="121" t="n">
+      <c r="F68" s="33" t="n">
         <v>763.7881165185184</v>
       </c>
     </row>
-    <row r="69" ht="16" customHeight="1">
-      <c r="A69" s="116" t="n">
+    <row r="69">
+      <c r="A69" s="29" t="n">
         <v>2024</v>
       </c>
-      <c r="B69" s="122" t="n">
+      <c r="B69" s="65" t="n">
         <v>82</v>
       </c>
-      <c r="C69" s="118" t="n">
+      <c r="C69" s="30" t="n">
         <v>1622.9</v>
       </c>
-      <c r="D69" s="123" t="n">
+      <c r="D69" s="73" t="n">
         <v>59631.35073</v>
       </c>
-      <c r="E69" s="120" t="n">
+      <c r="E69" s="32" t="n">
         <v>19.79146341463415</v>
       </c>
-      <c r="F69" s="121" t="n">
+      <c r="F69" s="33" t="n">
         <v>727.2115942682926</v>
       </c>
     </row>
-    <row r="70" ht="16" customHeight="1" thickBot="1">
-      <c r="A70" s="116" t="n">
+    <row r="70" ht="15" customHeight="1" thickBot="1">
+      <c r="A70" s="29" t="n">
         <v>2025</v>
       </c>
-      <c r="B70" s="124" t="n">
+      <c r="B70" s="66" t="n">
         <v>83</v>
       </c>
-      <c r="C70" s="125" t="n">
+      <c r="C70" s="67" t="n">
         <v>1635</v>
       </c>
-      <c r="D70" s="126" t="n">
+      <c r="D70" s="68" t="n">
         <v>60075.9495</v>
       </c>
-      <c r="E70" s="127" t="n">
+      <c r="E70" s="69" t="n">
         <v>19.69879518072289</v>
       </c>
-      <c r="F70" s="128" t="n">
+      <c r="F70" s="70" t="n">
         <v>723.8066204819277</v>
       </c>
     </row>
-    <row r="71" ht="16" customHeight="1">
-      <c r="A71" s="129" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="102" t="inlineStr">
         <is>
           <t xml:space="preserve"> r: revised</t>
         </is>
       </c>
-      <c r="B71" s="130" t="n"/>
-      <c r="C71" s="130" t="n"/>
-      <c r="D71" s="130" t="n"/>
-      <c r="E71" s="130" t="n"/>
-      <c r="F71" s="131" t="n"/>
-    </row>
-    <row r="72" ht="16" customHeight="1">
-      <c r="A72" s="132" t="inlineStr">
+      <c r="B71" s="103" t="n"/>
+      <c r="C71" s="103" t="n"/>
+      <c r="D71" s="103" t="n"/>
+      <c r="E71" s="103" t="n"/>
+      <c r="F71" s="104" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="105" t="inlineStr">
         <is>
           <t>*  Wheat equivalent.</t>
         </is>
       </c>
-      <c r="F72" s="133" t="n"/>
+      <c r="F72" s="106" t="n"/>
       <c r="G72" s="12" t="n"/>
     </row>
-    <row r="73" ht="16" customHeight="1" thickBot="1">
-      <c r="A73" s="134" t="inlineStr">
+    <row r="73" ht="15" customHeight="1" thickBot="1">
+      <c r="A73" s="107" t="inlineStr">
         <is>
           <t>SOURCE:  Canadian Grain Commission, Grain Elevators in Canada, August 2025</t>
         </is>
       </c>
-      <c r="B73" s="135" t="n"/>
-      <c r="C73" s="135" t="n"/>
-      <c r="D73" s="135" t="n"/>
-      <c r="E73" s="135" t="n"/>
-      <c r="F73" s="136" t="n"/>
-    </row>
-    <row r="74"/>
-    <row r="75" ht="16" customHeight="1">
-      <c r="A75" s="137" t="inlineStr">
+      <c r="B73" s="108" t="n"/>
+      <c r="C73" s="108" t="n"/>
+      <c r="D73" s="108" t="n"/>
+      <c r="E73" s="108" t="n"/>
+      <c r="F73" s="109" t="n"/>
+    </row>
+    <row r="75" ht="15" customHeight="1">
+      <c r="A75" s="71" t="inlineStr">
         <is>
           <t>Contact Us: Manitoba Agriculture, Foresight and Analysis;</t>
         </is>
       </c>
       <c r="B75" s="1" t="n"/>
-      <c r="E75" s="28" t="inlineStr">
+      <c r="E75" s="72" t="inlineStr">
         <is>
           <t>IndustryIntelligence@gov.mb.ca</t>
         </is>
@@ -3187,15 +3000,15 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="16.6640625" customWidth="1" min="1" max="1"/>
     <col width="13.5546875" customWidth="1" min="2" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="n"/>
-      <c r="B1" s="98" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Foresight and Analysis</t>
         </is>
@@ -3208,7 +3021,7 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2" ht="16" customHeight="1">
+    <row r="2">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="28" t="inlineStr">
         <is>
@@ -3234,8 +3047,8 @@
       <c r="H3" s="75" t="n"/>
       <c r="I3" s="75" t="n"/>
     </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="138" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
         <is>
           <t>Grain Storage Capacity,  Manitoba</t>
         </is>
@@ -3249,7 +3062,7 @@
       <c r="H4" s="75" t="n"/>
       <c r="I4" s="75" t="n"/>
     </row>
-    <row r="5" ht="16" customHeight="1" thickBot="1">
+    <row r="5" ht="15" customHeight="1" thickBot="1">
       <c r="A5" s="36" t="n"/>
       <c r="B5" s="36" t="n"/>
       <c r="C5" s="36" t="n"/>
@@ -3260,72 +3073,72 @@
       <c r="H5" s="75" t="n"/>
       <c r="I5" s="75" t="n"/>
     </row>
-    <row r="6" ht="16" customHeight="1" thickBot="1">
+    <row r="6" ht="15" customHeight="1" thickBot="1">
       <c r="A6" s="38" t="n"/>
-      <c r="B6" s="139" t="inlineStr">
+      <c r="B6" s="110" t="inlineStr">
         <is>
           <t>All Licensed Elevators</t>
         </is>
       </c>
-      <c r="C6" s="130" t="n"/>
-      <c r="D6" s="130" t="n"/>
-      <c r="E6" s="130" t="n"/>
-      <c r="F6" s="130" t="n"/>
-      <c r="G6" s="131" t="n"/>
+      <c r="C6" s="103" t="n"/>
+      <c r="D6" s="103" t="n"/>
+      <c r="E6" s="103" t="n"/>
+      <c r="F6" s="103" t="n"/>
+      <c r="G6" s="104" t="n"/>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
     </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="140" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>Kind of Elevator</t>
         </is>
       </c>
-      <c r="B7" s="141" t="inlineStr">
+      <c r="B7" s="111" t="inlineStr">
         <is>
           <t>2024 Capacity</t>
         </is>
       </c>
-      <c r="C7" s="142" t="n"/>
-      <c r="D7" s="105" t="n"/>
-      <c r="E7" s="141" t="inlineStr">
+      <c r="C7" s="112" t="n"/>
+      <c r="D7" s="101" t="n"/>
+      <c r="E7" s="111" t="inlineStr">
         <is>
           <t>2025 capacity</t>
         </is>
       </c>
-      <c r="F7" s="142" t="n"/>
-      <c r="G7" s="105" t="n"/>
+      <c r="F7" s="112" t="n"/>
+      <c r="G7" s="101" t="n"/>
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
     </row>
-    <row r="8" ht="16" customHeight="1" thickBot="1">
+    <row r="8" ht="15" customHeight="1" thickBot="1">
       <c r="A8" s="40" t="n"/>
-      <c r="B8" s="143" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="C8" s="144" t="inlineStr">
+      <c r="C8" s="42" t="inlineStr">
         <is>
           <t>000 tonnes</t>
         </is>
       </c>
-      <c r="D8" s="145" t="inlineStr">
+      <c r="D8" s="43" t="inlineStr">
         <is>
           <t>000 bushels*</t>
         </is>
       </c>
-      <c r="E8" s="143" t="inlineStr">
+      <c r="E8" s="41" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="F8" s="144" t="inlineStr">
+      <c r="F8" s="42" t="inlineStr">
         <is>
           <t>000 tonnes</t>
         </is>
       </c>
-      <c r="G8" s="146" t="inlineStr">
+      <c r="G8" s="44" t="inlineStr">
         <is>
           <t>000 bushels*</t>
         </is>
@@ -3333,141 +3146,141 @@
       <c r="H8" s="75" t="n"/>
       <c r="I8" s="75" t="n"/>
     </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="147" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="45" t="inlineStr">
         <is>
           <t xml:space="preserve">Terminal </t>
         </is>
       </c>
-      <c r="B9" s="148" t="n">
+      <c r="B9" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="149" t="n">
+      <c r="C9" s="47" t="n">
         <v>140.02</v>
       </c>
-      <c r="D9" s="150" t="n">
+      <c r="D9" s="48" t="n">
         <v>5144.894880000001</v>
       </c>
-      <c r="E9" s="148" t="n">
+      <c r="E9" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="151" t="n">
+      <c r="F9" s="49" t="n">
         <v>140</v>
       </c>
-      <c r="G9" s="152" t="n">
+      <c r="G9" s="50" t="n">
         <v>5144.16</v>
       </c>
       <c r="H9" s="75" t="n"/>
       <c r="I9" s="75" t="n"/>
     </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="153" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Process Elevators </t>
         </is>
       </c>
-      <c r="B10" s="154" t="n">
+      <c r="B10" s="52" t="n">
         <v>16</v>
       </c>
-      <c r="C10" s="155" t="n">
+      <c r="C10" s="53" t="n">
         <v>129.9</v>
       </c>
-      <c r="D10" s="156" t="n">
+      <c r="D10" s="54" t="n">
         <v>4773.00663</v>
       </c>
-      <c r="E10" s="154" t="n">
+      <c r="E10" s="52" t="n">
         <v>17</v>
       </c>
-      <c r="F10" s="157" t="n">
+      <c r="F10" s="55" t="n">
         <v>132.3</v>
       </c>
-      <c r="G10" s="152" t="n">
+      <c r="G10" s="50" t="n">
         <v>4860.3051</v>
       </c>
       <c r="H10" s="5" t="n"/>
       <c r="I10" s="5" t="n"/>
     </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="153" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Primary </t>
         </is>
       </c>
-      <c r="B11" s="158" t="n">
+      <c r="B11" s="56" t="n">
         <v>82</v>
       </c>
-      <c r="C11" s="159" t="n">
+      <c r="C11" s="57" t="n">
         <v>1622.9</v>
       </c>
-      <c r="D11" s="156" t="n">
+      <c r="D11" s="54" t="n">
         <v>59631.35073</v>
       </c>
-      <c r="E11" s="158" t="n">
+      <c r="E11" s="56" t="n">
         <v>83</v>
       </c>
-      <c r="F11" s="160" t="n">
+      <c r="F11" s="58" t="n">
         <v>1635</v>
       </c>
-      <c r="G11" s="152" t="n">
+      <c r="G11" s="50" t="n">
         <v>60076</v>
       </c>
       <c r="H11" s="5" t="n"/>
       <c r="I11" s="5" t="n"/>
     </row>
-    <row r="12" ht="16" customHeight="1" thickBot="1">
-      <c r="A12" s="161" t="inlineStr">
+    <row r="12" ht="15" customHeight="1" thickBot="1">
+      <c r="A12" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">TOTAL - Licensed </t>
         </is>
       </c>
-      <c r="B12" s="162" t="n">
+      <c r="B12" s="60" t="n">
         <v>99</v>
       </c>
-      <c r="C12" s="163" t="n">
+      <c r="C12" s="61" t="n">
         <v>1892.82</v>
       </c>
-      <c r="D12" s="164" t="n">
+      <c r="D12" s="62" t="n">
         <v>69549.25224</v>
       </c>
-      <c r="E12" s="162" t="n">
+      <c r="E12" s="60" t="n">
         <v>101</v>
       </c>
-      <c r="F12" s="165" t="n">
+      <c r="F12" s="63" t="n">
         <v>1907.3</v>
       </c>
-      <c r="G12" s="166" t="n">
+      <c r="G12" s="64" t="n">
         <v>70080.4651</v>
       </c>
       <c r="H12" s="5" t="n"/>
       <c r="I12" s="5" t="n"/>
     </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="147" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="45" t="inlineStr">
         <is>
           <t>*  Wheat equivalent.</t>
         </is>
       </c>
-      <c r="B13" s="130" t="n"/>
-      <c r="C13" s="130" t="n"/>
-      <c r="D13" s="130" t="n"/>
-      <c r="E13" s="130" t="n"/>
-      <c r="F13" s="130" t="n"/>
-      <c r="G13" s="131" t="n"/>
+      <c r="B13" s="103" t="n"/>
+      <c r="C13" s="103" t="n"/>
+      <c r="D13" s="103" t="n"/>
+      <c r="E13" s="103" t="n"/>
+      <c r="F13" s="103" t="n"/>
+      <c r="G13" s="104" t="n"/>
       <c r="H13" s="5" t="n"/>
       <c r="I13" s="5" t="n"/>
     </row>
-    <row r="14" ht="16" customHeight="1" thickBot="1">
-      <c r="A14" s="167" t="inlineStr">
+    <row r="14" ht="15" customHeight="1" thickBot="1">
+      <c r="A14" s="113" t="inlineStr">
         <is>
           <t>SOURCE:  Canadian Grain Commission, Grain Elevators in Canada, August 2024 and 2025</t>
         </is>
       </c>
-      <c r="B14" s="135" t="n"/>
-      <c r="C14" s="135" t="n"/>
-      <c r="D14" s="135" t="n"/>
-      <c r="E14" s="135" t="n"/>
-      <c r="F14" s="135" t="n"/>
-      <c r="G14" s="136" t="n"/>
+      <c r="B14" s="108" t="n"/>
+      <c r="C14" s="108" t="n"/>
+      <c r="D14" s="108" t="n"/>
+      <c r="E14" s="108" t="n"/>
+      <c r="F14" s="108" t="n"/>
+      <c r="G14" s="109" t="n"/>
       <c r="H14" s="5" t="n"/>
       <c r="I14" s="5" t="n"/>
     </row>
@@ -3482,15 +3295,15 @@
       <c r="H15" s="5" t="n"/>
       <c r="I15" s="5" t="n"/>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="137" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Contact Us: Manitoba Agriculture, Foresight and Analysis;</t>
         </is>
       </c>
       <c r="B16" s="1" t="n"/>
       <c r="C16" s="75" t="n"/>
-      <c r="D16" s="28" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>IndustryIntelligence@gov.mb.ca</t>
         </is>

</xml_diff>

<commit_message>
MB elevator workbook: set explicit 18pt height on every populated row (rows without explicit heights were falling back to ~12.75); fonts untouched
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mb_primary_elevator_capacity_2025.xlsx
+++ b/textbook_examples/mb_primary_elevator_capacity_2025.xlsx
@@ -1482,7 +1482,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K75"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col width="6.5546875" customWidth="1" style="75" min="1" max="1"/>
     <col width="10.88671875" customWidth="1" style="75" min="2" max="2"/>
@@ -1497,7 +1497,7 @@
     <col width="9.109375" customWidth="1" style="75" min="12" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="C1" s="9" t="inlineStr">
         <is>
@@ -1507,7 +1507,7 @@
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="C2" s="28" t="inlineStr">
         <is>
@@ -1542,7 +1542,7 @@
     <row r="5" ht="15" customHeight="1" thickBot="1">
       <c r="A5" s="4" t="n"/>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="18" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Year</t>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="F6" s="101" t="n"/>
     </row>
-    <row r="7" ht="15" customHeight="1">
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" s="16" t="n"/>
       <c r="B7" s="17" t="n"/>
       <c r="C7" s="18" t="inlineStr">
@@ -1595,7 +1595,7 @@
       <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="n"/>
     </row>
-    <row r="8" ht="15" customHeight="1">
+    <row r="8" ht="18" customHeight="1">
       <c r="A8" s="20" t="n">
         <v>1963</v>
       </c>
@@ -1620,7 +1620,7 @@
       <c r="J8" s="9" t="n"/>
       <c r="K8" s="9" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="18" customHeight="1">
       <c r="A9" s="24" t="n">
         <v>1964</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>73.8</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="18" customHeight="1">
       <c r="A10" s="24" t="n">
         <v>1965</v>
       </c>
@@ -1660,7 +1660,7 @@
         <v>75.40000000000001</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="18" customHeight="1">
       <c r="A11" s="24" t="n">
         <v>1966</v>
       </c>
@@ -1685,7 +1685,7 @@
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="18" customHeight="1">
       <c r="A12" s="24" t="n">
         <v>1967</v>
       </c>
@@ -1710,7 +1710,7 @@
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="18" customHeight="1">
       <c r="A13" s="24" t="n">
         <v>1968</v>
       </c>
@@ -1735,7 +1735,7 @@
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" ht="18" customHeight="1">
       <c r="A14" s="24" t="n">
         <v>1969</v>
       </c>
@@ -1760,7 +1760,7 @@
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="18" customHeight="1">
       <c r="A15" s="24" t="n">
         <v>1970</v>
       </c>
@@ -1785,7 +1785,7 @@
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="18" customHeight="1">
       <c r="A16" s="24" t="n">
         <v>1971</v>
       </c>
@@ -1810,7 +1810,7 @@
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="18" customHeight="1">
       <c r="A17" s="24" t="n">
         <v>1972</v>
       </c>
@@ -1835,7 +1835,7 @@
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" ht="18" customHeight="1">
       <c r="A18" s="24" t="n">
         <v>1973</v>
       </c>
@@ -1860,7 +1860,7 @@
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" ht="18" customHeight="1">
       <c r="A19" s="24" t="n">
         <v>1974</v>
       </c>
@@ -1885,7 +1885,7 @@
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
     </row>
-    <row r="20">
+    <row r="20" ht="18" customHeight="1">
       <c r="A20" s="24" t="n">
         <v>1975</v>
       </c>
@@ -1910,7 +1910,7 @@
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="6" t="n"/>
     </row>
-    <row r="21">
+    <row r="21" ht="18" customHeight="1">
       <c r="A21" s="24" t="n">
         <v>1976</v>
       </c>
@@ -1935,7 +1935,7 @@
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
     </row>
-    <row r="22" ht="15" customHeight="1">
+    <row r="22" ht="18" customHeight="1">
       <c r="A22" s="24" t="n">
         <v>1977</v>
       </c>
@@ -1960,7 +1960,7 @@
       <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
     </row>
-    <row r="23">
+    <row r="23" ht="18" customHeight="1">
       <c r="A23" s="24" t="n">
         <v>1978</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>100.2</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="18" customHeight="1">
       <c r="A24" s="24" t="n">
         <v>1979</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>103.7</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="18" customHeight="1">
       <c r="A25" s="24" t="n">
         <v>1980</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>106.4</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="18" customHeight="1">
       <c r="A26" s="24" t="n">
         <v>1981</v>
       </c>
@@ -2045,7 +2045,7 @@
       <c r="J26" s="10" t="n"/>
       <c r="K26" s="10" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="18" customHeight="1">
       <c r="A27" s="24" t="n">
         <v>1982</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>116.3</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="18" customHeight="1">
       <c r="A28" s="24" t="n">
         <v>1983</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>116.8</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="18" customHeight="1">
       <c r="A29" s="24" t="n">
         <v>1984</v>
       </c>
@@ -2105,7 +2105,7 @@
         <v>134.5</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="18" customHeight="1">
       <c r="A30" s="24" t="n">
         <v>1985</v>
       </c>
@@ -2125,7 +2125,7 @@
         <v>135.5</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="18" customHeight="1">
       <c r="A31" s="24" t="n">
         <v>1986</v>
       </c>
@@ -2145,7 +2145,7 @@
         <v>140.3</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="18" customHeight="1">
       <c r="A32" s="24" t="n">
         <v>1987</v>
       </c>
@@ -2165,7 +2165,7 @@
         <v>141.1</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="18" customHeight="1">
       <c r="A33" s="24" t="n">
         <v>1988</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>142.9</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="18" customHeight="1">
       <c r="A34" s="24" t="n">
         <v>1989</v>
       </c>
@@ -2205,7 +2205,7 @@
         <v>144.8</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="18" customHeight="1">
       <c r="A35" s="24" t="n">
         <v>1990</v>
       </c>
@@ -2225,7 +2225,7 @@
         <v>154.5</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="18" customHeight="1">
       <c r="A36" s="24" t="n">
         <v>1991</v>
       </c>
@@ -2245,7 +2245,7 @@
         <v>155.8</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="18" customHeight="1">
       <c r="A37" s="24" t="n">
         <v>1992</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>155.9</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="18" customHeight="1">
       <c r="A38" s="24" t="n">
         <v>1993</v>
       </c>
@@ -2285,7 +2285,7 @@
         <v>156.8</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="18" customHeight="1">
       <c r="A39" s="24" t="n">
         <v>1994</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="18" customHeight="1">
       <c r="A40" s="24" t="n">
         <v>1995</v>
       </c>
@@ -2325,7 +2325,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="18" customHeight="1">
       <c r="A41" s="24" t="n">
         <v>1996</v>
       </c>
@@ -2345,7 +2345,7 @@
         <v>173.8</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="18" customHeight="1">
       <c r="A42" s="24" t="n">
         <v>1997</v>
       </c>
@@ -2365,7 +2365,7 @@
         <v>176.2</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="18" customHeight="1">
       <c r="A43" s="24" t="n">
         <v>1998</v>
       </c>
@@ -2385,7 +2385,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="18" customHeight="1">
       <c r="A44" s="24" t="n">
         <v>1999</v>
       </c>
@@ -2405,7 +2405,7 @@
         <v>206.4</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="18" customHeight="1">
       <c r="A45" s="24" t="n">
         <v>2000</v>
       </c>
@@ -2425,7 +2425,7 @@
         <v>234.5</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="18" customHeight="1">
       <c r="A46" s="24" t="n">
         <v>2001</v>
       </c>
@@ -2445,7 +2445,7 @@
         <v>276.2</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="18" customHeight="1">
       <c r="A47" s="24" t="n">
         <v>2002</v>
       </c>
@@ -2465,7 +2465,7 @@
         <v>364.6</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="18" customHeight="1">
       <c r="A48" s="24" t="n">
         <v>2003</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>393.2</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="18" customHeight="1">
       <c r="A49" s="24" t="n">
         <v>2004</v>
       </c>
@@ -2505,7 +2505,7 @@
         <v>433.6</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="18" customHeight="1">
       <c r="A50" s="24" t="n">
         <v>2005</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>459.3</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="18" customHeight="1">
       <c r="A51" s="24" t="n">
         <v>2006</v>
       </c>
@@ -2545,7 +2545,7 @@
         <v>468.6</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="18" customHeight="1">
       <c r="A52" s="24" t="n">
         <v>2007</v>
       </c>
@@ -2565,7 +2565,7 @@
         <v>458.9</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="18" customHeight="1">
       <c r="A53" s="24" t="n">
         <v>2008</v>
       </c>
@@ -2585,7 +2585,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="18" customHeight="1">
       <c r="A54" s="24" t="n">
         <v>2009</v>
       </c>
@@ -2605,7 +2605,7 @@
         <v>506.1662169863014</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="18" customHeight="1">
       <c r="A55" s="24" t="n">
         <v>2010</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>503.2400976623376</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="18" customHeight="1">
       <c r="A56" s="24" t="n">
         <v>2011</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>555.7249016470588</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="18" customHeight="1">
       <c r="A57" s="24" t="n">
         <v>2012</v>
       </c>
@@ -2665,7 +2665,7 @@
         <v>502.369614</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" ht="18" customHeight="1">
       <c r="A58" s="24" t="n">
         <v>2013</v>
       </c>
@@ -2685,7 +2685,7 @@
         <v>490.5860710112359</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="18" customHeight="1">
       <c r="A59" s="24" t="n">
         <v>2014</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>602.4626897560976</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="18" customHeight="1">
       <c r="A60" s="24" t="n">
         <v>2015</v>
       </c>
@@ -2725,7 +2725,7 @@
         <v>597.117558</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="18" customHeight="1">
       <c r="A61" s="24" t="n">
         <v>2016</v>
       </c>
@@ -2745,7 +2745,7 @@
         <v>670.4032419512196</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="24" t="n">
         <v>2017</v>
       </c>
@@ -2765,7 +2765,7 @@
         <v>697.471108571429</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="18" customHeight="1">
       <c r="A63" s="24" t="n">
         <v>2018</v>
       </c>
@@ -2785,7 +2785,7 @@
         <v>699.1</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="18" customHeight="1">
       <c r="A64" s="29" t="n">
         <v>2019</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>698.4385976470588</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="18" customHeight="1">
       <c r="A65" s="29" t="n">
         <v>2020</v>
       </c>
@@ -2825,7 +2825,7 @@
         <v>717.4376674698794</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" ht="18" customHeight="1">
       <c r="A66" s="29" t="n">
         <v>2021</v>
       </c>
@@ -2845,7 +2845,7 @@
         <v>744.89274</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="18" customHeight="1">
       <c r="A67" s="29" t="n">
         <v>2022</v>
       </c>
@@ -2865,7 +2865,7 @@
         <v>744.6132939759035</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="18" customHeight="1">
       <c r="A68" s="29" t="n">
         <v>2023</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>763.7881165185184</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" ht="18" customHeight="1">
       <c r="A69" s="29" t="n">
         <v>2024</v>
       </c>
@@ -2905,7 +2905,7 @@
         <v>727.2115942682926</v>
       </c>
     </row>
-    <row r="70" ht="15" customHeight="1" thickBot="1">
+    <row r="70" ht="18" customHeight="1" thickBot="1">
       <c r="A70" s="29" t="n">
         <v>2025</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>723.8066204819277</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" ht="18" customHeight="1">
       <c r="A71" s="102" t="inlineStr">
         <is>
           <t xml:space="preserve"> r: revised</t>
@@ -2937,7 +2937,7 @@
       <c r="E71" s="103" t="n"/>
       <c r="F71" s="104" t="n"/>
     </row>
-    <row r="72">
+    <row r="72" ht="18" customHeight="1">
       <c r="A72" s="105" t="inlineStr">
         <is>
           <t>*  Wheat equivalent.</t>
@@ -2946,7 +2946,7 @@
       <c r="F72" s="106" t="n"/>
       <c r="G72" s="12" t="n"/>
     </row>
-    <row r="73" ht="15" customHeight="1" thickBot="1">
+    <row r="73" ht="18" customHeight="1" thickBot="1">
       <c r="A73" s="107" t="inlineStr">
         <is>
           <t>SOURCE:  Canadian Grain Commission, Grain Elevators in Canada, August 2025</t>
@@ -2958,7 +2958,8 @@
       <c r="E73" s="108" t="n"/>
       <c r="F73" s="109" t="n"/>
     </row>
-    <row r="75" ht="15" customHeight="1">
+    <row r="74"/>
+    <row r="75" ht="18" customHeight="1">
       <c r="A75" s="71" t="inlineStr">
         <is>
           <t>Contact Us: Manitoba Agriculture, Foresight and Analysis;</t>
@@ -3000,13 +3001,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col width="16.6640625" customWidth="1" min="1" max="1"/>
     <col width="13.5546875" customWidth="1" min="2" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="9" t="inlineStr">
         <is>
@@ -3021,7 +3022,7 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="28" t="inlineStr">
         <is>
@@ -3047,7 +3048,7 @@
       <c r="H3" s="75" t="n"/>
       <c r="I3" s="75" t="n"/>
     </row>
-    <row r="4">
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="35" t="inlineStr">
         <is>
           <t>Grain Storage Capacity,  Manitoba</t>
@@ -3073,7 +3074,7 @@
       <c r="H5" s="75" t="n"/>
       <c r="I5" s="75" t="n"/>
     </row>
-    <row r="6" ht="15" customHeight="1" thickBot="1">
+    <row r="6" ht="18" customHeight="1" thickBot="1">
       <c r="A6" s="38" t="n"/>
       <c r="B6" s="110" t="inlineStr">
         <is>
@@ -3088,7 +3089,7 @@
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" s="39" t="inlineStr">
         <is>
           <t>Kind of Elevator</t>
@@ -3111,7 +3112,7 @@
       <c r="H7" s="9" t="n"/>
       <c r="I7" s="9" t="n"/>
     </row>
-    <row r="8" ht="15" customHeight="1" thickBot="1">
+    <row r="8" ht="18" customHeight="1" thickBot="1">
       <c r="A8" s="40" t="n"/>
       <c r="B8" s="41" t="inlineStr">
         <is>
@@ -3146,7 +3147,7 @@
       <c r="H8" s="75" t="n"/>
       <c r="I8" s="75" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="18" customHeight="1">
       <c r="A9" s="45" t="inlineStr">
         <is>
           <t xml:space="preserve">Terminal </t>
@@ -3173,7 +3174,7 @@
       <c r="H9" s="75" t="n"/>
       <c r="I9" s="75" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="18" customHeight="1">
       <c r="A10" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Process Elevators </t>
@@ -3200,7 +3201,7 @@
       <c r="H10" s="5" t="n"/>
       <c r="I10" s="5" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="18" customHeight="1">
       <c r="A11" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Primary </t>
@@ -3227,7 +3228,7 @@
       <c r="H11" s="5" t="n"/>
       <c r="I11" s="5" t="n"/>
     </row>
-    <row r="12" ht="15" customHeight="1" thickBot="1">
+    <row r="12" ht="18" customHeight="1" thickBot="1">
       <c r="A12" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">TOTAL - Licensed </t>
@@ -3254,7 +3255,7 @@
       <c r="H12" s="5" t="n"/>
       <c r="I12" s="5" t="n"/>
     </row>
-    <row r="13">
+    <row r="13" ht="18" customHeight="1">
       <c r="A13" s="45" t="inlineStr">
         <is>
           <t>*  Wheat equivalent.</t>
@@ -3269,7 +3270,7 @@
       <c r="H13" s="5" t="n"/>
       <c r="I13" s="5" t="n"/>
     </row>
-    <row r="14" ht="15" customHeight="1" thickBot="1">
+    <row r="14" ht="18" customHeight="1" thickBot="1">
       <c r="A14" s="113" t="inlineStr">
         <is>
           <t>SOURCE:  Canadian Grain Commission, Grain Elevators in Canada, August 2024 and 2025</t>
@@ -3295,7 +3296,7 @@
       <c r="H15" s="5" t="n"/>
       <c r="I15" s="5" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="18" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Contact Us: Manitoba Agriculture, Foresight and Analysis;</t>

</xml_diff>